<commit_message>
Add match: T20 vs Hollywoodbets Dolphins, 2026-10-04
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/raw/Mayes_Bowling_Batting.xlsx
+++ b/backend/data/raw/Mayes_Bowling_Batting.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T216"/>
+  <dimension ref="A1:T234"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="10.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="20.44140625" bestFit="1" customWidth="1" min="2" max="2"/>
@@ -21073,6 +21073,1591 @@
         </is>
       </c>
     </row>
+    <row r="217">
+      <c r="A217" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>Hollywoodbets Dolphins</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>Polokwane</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>End 2</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>B Parsons</t>
+        </is>
+      </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>Left</t>
+        </is>
+      </c>
+      <c r="K217" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="L217" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M217" t="inlineStr">
+        <is>
+          <t>Leg Stump</t>
+        </is>
+      </c>
+      <c r="N217" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="O217" t="n">
+        <v>1</v>
+      </c>
+      <c r="P217" t="inlineStr">
+        <is>
+          <t>Leg Bye</t>
+        </is>
+      </c>
+      <c r="Q217" t="inlineStr">
+        <is>
+          <t>Cover</t>
+        </is>
+      </c>
+      <c r="R217" t="inlineStr">
+        <is>
+          <t>Back Foot Flick</t>
+        </is>
+      </c>
+      <c r="S217" t="inlineStr">
+        <is>
+          <t>Miss</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>Hollywoodbets Dolphins</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>Polokwane</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>End 2</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>R Pillay</t>
+        </is>
+      </c>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K218" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="L218" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M218" t="inlineStr">
+        <is>
+          <t>Wide</t>
+        </is>
+      </c>
+      <c r="N218" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="O218" t="n">
+        <v>0</v>
+      </c>
+      <c r="P218" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="R218" t="inlineStr">
+        <is>
+          <t>Cut</t>
+        </is>
+      </c>
+      <c r="S218" t="inlineStr">
+        <is>
+          <t>Miss</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>Hollywoodbets Dolphins</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>Polokwane</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>End 2</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>R Pillay</t>
+        </is>
+      </c>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K219" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="L219" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M219" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="N219" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="O219" t="n">
+        <v>0</v>
+      </c>
+      <c r="P219" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="R219" t="inlineStr">
+        <is>
+          <t>Off Drive</t>
+        </is>
+      </c>
+      <c r="S219" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>Hollywoodbets Dolphins</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>Polokwane</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>End 2</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>R Pillay</t>
+        </is>
+      </c>
+      <c r="J220" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K220" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="L220" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M220" t="inlineStr">
+        <is>
+          <t>Off Stump</t>
+        </is>
+      </c>
+      <c r="N220" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="O220" t="n">
+        <v>0</v>
+      </c>
+      <c r="P220" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="R220" t="inlineStr">
+        <is>
+          <t>Hack</t>
+        </is>
+      </c>
+      <c r="S220" t="inlineStr">
+        <is>
+          <t>Miss</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>Hollywoodbets Dolphins</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>Polokwane</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>End 2</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>R Pillay</t>
+        </is>
+      </c>
+      <c r="J221" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K221" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="L221" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M221" t="inlineStr">
+        <is>
+          <t>Leg Stump</t>
+        </is>
+      </c>
+      <c r="N221" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="O221" t="n">
+        <v>1</v>
+      </c>
+      <c r="P221" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="Q221" t="inlineStr">
+        <is>
+          <t>Mid On</t>
+        </is>
+      </c>
+      <c r="R221" t="inlineStr">
+        <is>
+          <t>Pull</t>
+        </is>
+      </c>
+      <c r="S221" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>Hollywoodbets Dolphins</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>Polokwane</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>End 2</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>B Parsons</t>
+        </is>
+      </c>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>Left</t>
+        </is>
+      </c>
+      <c r="K222" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="L222" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M222" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="N222" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="O222" t="n">
+        <v>0</v>
+      </c>
+      <c r="P222" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="R222" t="inlineStr">
+        <is>
+          <t>Cover Drive</t>
+        </is>
+      </c>
+      <c r="S222" t="inlineStr">
+        <is>
+          <t>Miss</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>Hollywoodbets Dolphins</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>Polokwane</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>End 2</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>J Smith</t>
+        </is>
+      </c>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K223" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="L223" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M223" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="N223" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="O223" t="n">
+        <v>0</v>
+      </c>
+      <c r="P223" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="R223" t="inlineStr">
+        <is>
+          <t>Front Foot Defense</t>
+        </is>
+      </c>
+      <c r="S223" t="inlineStr">
+        <is>
+          <t>Miss</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>Hollywoodbets Dolphins</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>Polokwane</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>End 2</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>J Smith</t>
+        </is>
+      </c>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K224" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="L224" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M224" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="N224" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="O224" t="n">
+        <v>1</v>
+      </c>
+      <c r="P224" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="R224" t="inlineStr">
+        <is>
+          <t>Front Foot Defense</t>
+        </is>
+      </c>
+      <c r="S224" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>Hollywoodbets Dolphins</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>Polokwane</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>End 2</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>R Pillay</t>
+        </is>
+      </c>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K225" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="L225" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M225" t="inlineStr">
+        <is>
+          <t>Off Stump</t>
+        </is>
+      </c>
+      <c r="N225" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="O225" t="n">
+        <v>1</v>
+      </c>
+      <c r="P225" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="R225" t="inlineStr">
+        <is>
+          <t>Off Drive</t>
+        </is>
+      </c>
+      <c r="S225" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>Hollywoodbets Dolphins</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>Polokwane</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>End 2</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>J Smith</t>
+        </is>
+      </c>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K226" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="L226" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M226" t="inlineStr">
+        <is>
+          <t>Leg Stump</t>
+        </is>
+      </c>
+      <c r="N226" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="O226" t="n">
+        <v>0</v>
+      </c>
+      <c r="P226" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="R226" t="inlineStr">
+        <is>
+          <t>Pull</t>
+        </is>
+      </c>
+      <c r="S226" t="inlineStr">
+        <is>
+          <t>Miss</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>Hollywoodbets Dolphins</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>Polokwane</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>End 2</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>J Smith</t>
+        </is>
+      </c>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K227" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="L227" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M227" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="N227" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="O227" t="inlineStr">
+        <is>
+          <t>Wicket</t>
+        </is>
+      </c>
+      <c r="P227" t="inlineStr">
+        <is>
+          <t>Caught</t>
+        </is>
+      </c>
+      <c r="Q227" t="inlineStr">
+        <is>
+          <t>Extra Cover</t>
+        </is>
+      </c>
+      <c r="R227" t="inlineStr">
+        <is>
+          <t>Cover Drive</t>
+        </is>
+      </c>
+      <c r="S227" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+      <c r="T227" t="inlineStr">
+        <is>
+          <t>Caught at Extra Cover</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>Hollywoodbets Dolphins</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>Polokwane</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>End 2</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>H Viljoen</t>
+        </is>
+      </c>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K228" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="L228" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M228" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="N228" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="O228" t="n">
+        <v>0</v>
+      </c>
+      <c r="P228" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="R228" t="inlineStr">
+        <is>
+          <t>Back Foot Defense</t>
+        </is>
+      </c>
+      <c r="S228" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>Hollywoodbets Dolphins</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>Polokwane</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>End 2</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>H Viljoen</t>
+        </is>
+      </c>
+      <c r="J229" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K229" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="L229" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M229" t="inlineStr">
+        <is>
+          <t>Middle Stump</t>
+        </is>
+      </c>
+      <c r="N229" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="O229" t="n">
+        <v>0</v>
+      </c>
+      <c r="P229" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="R229" t="inlineStr">
+        <is>
+          <t>Back Foot Defense</t>
+        </is>
+      </c>
+      <c r="S229" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>Hollywoodbets Dolphins</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>Polokwane</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>End 2</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>H Viljoen</t>
+        </is>
+      </c>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K230" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="L230" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M230" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="N230" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="O230" t="n">
+        <v>1</v>
+      </c>
+      <c r="P230" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="R230" t="inlineStr">
+        <is>
+          <t>On Drive</t>
+        </is>
+      </c>
+      <c r="S230" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>Hollywoodbets Dolphins</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>Polokwane</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>End 2</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>R Pillay</t>
+        </is>
+      </c>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K231" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="L231" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M231" t="inlineStr">
+        <is>
+          <t>Middle Stump</t>
+        </is>
+      </c>
+      <c r="N231" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="O231" t="n">
+        <v>1</v>
+      </c>
+      <c r="P231" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="Q231" t="inlineStr">
+        <is>
+          <t>Square Leg</t>
+        </is>
+      </c>
+      <c r="R231" t="inlineStr">
+        <is>
+          <t>Pull</t>
+        </is>
+      </c>
+      <c r="S231" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>Hollywoodbets Dolphins</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>Polokwane</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>End 2</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>H Viljoen</t>
+        </is>
+      </c>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K232" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="L232" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M232" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="N232" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="O232" t="n">
+        <v>1</v>
+      </c>
+      <c r="P232" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="Q232" t="inlineStr">
+        <is>
+          <t>Third Man</t>
+        </is>
+      </c>
+      <c r="R232" t="inlineStr">
+        <is>
+          <t>Guide</t>
+        </is>
+      </c>
+      <c r="S232" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>Hollywoodbets Dolphins</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>Polokwane</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>End 2</t>
+        </is>
+      </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>R Pillay</t>
+        </is>
+      </c>
+      <c r="J233" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K233" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="L233" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M233" t="inlineStr">
+        <is>
+          <t>Middle Stump</t>
+        </is>
+      </c>
+      <c r="N233" t="inlineStr">
+        <is>
+          <t>Yorker</t>
+        </is>
+      </c>
+      <c r="O233" t="n">
+        <v>0</v>
+      </c>
+      <c r="P233" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="R233" t="inlineStr">
+        <is>
+          <t>Dig Out</t>
+        </is>
+      </c>
+      <c r="S233" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>Hollywoodbets Dolphins</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>Polokwane</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>End 2</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>R Pillay</t>
+        </is>
+      </c>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K234" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="L234" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M234" t="inlineStr">
+        <is>
+          <t>Middle Stump</t>
+        </is>
+      </c>
+      <c r="N234" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="O234" t="n">
+        <v>4</v>
+      </c>
+      <c r="P234" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="Q234" t="inlineStr">
+        <is>
+          <t>Mid On</t>
+        </is>
+      </c>
+      <c r="R234" t="inlineStr">
+        <is>
+          <t>Lofted On Drive</t>
+        </is>
+      </c>
+      <c r="S234" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:S191">
     <sortState ref="A2:S191">
@@ -21089,7 +22674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q75"/>
+  <dimension ref="A1:Q77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="20.44140625" bestFit="1" customWidth="1" min="2" max="2"/>
@@ -27038,6 +28623,156 @@
         </is>
       </c>
       <c r="Q75" t="inlineStr">
+        <is>
+          <t>Miss</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Hollywoodbets Dolphins</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Polokwane</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="H76" t="n">
+        <v>7</v>
+      </c>
+      <c r="I76" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>T Luus</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>Wide</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>Cut</t>
+        </is>
+      </c>
+      <c r="N76" t="n">
+        <v>0</v>
+      </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="Q76" t="inlineStr">
+        <is>
+          <t>Miss</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Hollywoodbets Dolphins</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Polokwane</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="H77" t="n">
+        <v>7</v>
+      </c>
+      <c r="I77" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>T Luus</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>Leg Stump</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>Flick</t>
+        </is>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>Wicket</t>
+        </is>
+      </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>LBW</t>
+        </is>
+      </c>
+      <c r="Q77" t="inlineStr">
         <is>
           <t>Miss</t>
         </is>

</xml_diff>

<commit_message>
Show DNB when Thomas didn't bat or bowl in a match
A match where he only bowled (or only batted) previously just showed
the one discipline's figures with no indication the other was ever
considered - the Northern Cape Heat T20 (bowling only) made this
ambiguous rather than informative. The Home page's "most recent game"
panel, the match list chips, and the match detail view now all show
"DNB" for whichever discipline has no innings recorded for that match.

Also includes the Northern Cape Heat match data itself (bowling only,
2026-10-13) that prompted this.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/raw/Mayes_Bowling_Batting.xlsx
+++ b/backend/data/raw/Mayes_Bowling_Batting.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T234"/>
+  <dimension ref="A1:T258"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="10.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="20.44140625" bestFit="1" customWidth="1" min="2" max="2"/>
@@ -22653,6 +22653,2167 @@
         </is>
       </c>
       <c r="S234" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>Northern Cape Heat</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>Kimberley Oval</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>End 1</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>S Stolk</t>
+        </is>
+      </c>
+      <c r="J235" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K235" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L235" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M235" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="N235" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="O235" t="n">
+        <v>1</v>
+      </c>
+      <c r="P235" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="Q235" t="inlineStr">
+        <is>
+          <t>Third Man</t>
+        </is>
+      </c>
+      <c r="R235" t="inlineStr">
+        <is>
+          <t>Guide</t>
+        </is>
+      </c>
+      <c r="S235" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>Northern Cape Heat</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>Kimberley Oval</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>End 1</t>
+        </is>
+      </c>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I236" t="inlineStr">
+        <is>
+          <t>L Doherty</t>
+        </is>
+      </c>
+      <c r="J236" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K236" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L236" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M236" t="inlineStr">
+        <is>
+          <t>Leg Stump</t>
+        </is>
+      </c>
+      <c r="N236" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="O236" t="n">
+        <v>1</v>
+      </c>
+      <c r="P236" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="Q236" t="inlineStr">
+        <is>
+          <t>Square Leg</t>
+        </is>
+      </c>
+      <c r="R236" t="inlineStr">
+        <is>
+          <t>Back Foot Punch</t>
+        </is>
+      </c>
+      <c r="S236" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>Northern Cape Heat</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>Kimberley Oval</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>End 1</t>
+        </is>
+      </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>S Stolk</t>
+        </is>
+      </c>
+      <c r="J237" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K237" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L237" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M237" t="inlineStr">
+        <is>
+          <t>Off Stump</t>
+        </is>
+      </c>
+      <c r="N237" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="O237" t="n">
+        <v>4</v>
+      </c>
+      <c r="P237" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="Q237" t="inlineStr">
+        <is>
+          <t>Third Man</t>
+        </is>
+      </c>
+      <c r="R237" t="inlineStr">
+        <is>
+          <t>Back Foot Defense</t>
+        </is>
+      </c>
+      <c r="S237" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>Northern Cape Heat</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>Kimberley Oval</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>End 1</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>S Stolk</t>
+        </is>
+      </c>
+      <c r="J238" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K238" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L238" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M238" t="inlineStr">
+        <is>
+          <t>Wide</t>
+        </is>
+      </c>
+      <c r="N238" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="O238" t="n">
+        <v>1</v>
+      </c>
+      <c r="P238" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="Q238" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="R238" t="inlineStr">
+        <is>
+          <t>Cut</t>
+        </is>
+      </c>
+      <c r="S238" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>Northern Cape Heat</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>Kimberley Oval</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>End 1</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I239" t="inlineStr">
+        <is>
+          <t>L Doherty</t>
+        </is>
+      </c>
+      <c r="J239" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K239" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L239" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M239" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="N239" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="O239" t="n">
+        <v>0</v>
+      </c>
+      <c r="P239" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="R239" t="inlineStr">
+        <is>
+          <t>Back Foot Defense</t>
+        </is>
+      </c>
+      <c r="S239" t="inlineStr">
+        <is>
+          <t>Miss</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>Northern Cape Heat</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>Kimberley Oval</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>End 1</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>L Doherty</t>
+        </is>
+      </c>
+      <c r="J240" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K240" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L240" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M240" t="inlineStr">
+        <is>
+          <t>Wide</t>
+        </is>
+      </c>
+      <c r="N240" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="O240" t="n">
+        <v>1</v>
+      </c>
+      <c r="P240" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="Q240" t="inlineStr">
+        <is>
+          <t>Mid Off</t>
+        </is>
+      </c>
+      <c r="R240" t="inlineStr">
+        <is>
+          <t>Off Drive</t>
+        </is>
+      </c>
+      <c r="S240" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>Northern Cape Heat</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>Kimberley Oval</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>End 1</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>L Doherty</t>
+        </is>
+      </c>
+      <c r="J241" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K241" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="L241" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M241" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="N241" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="O241" t="n">
+        <v>1</v>
+      </c>
+      <c r="P241" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="Q241" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="R241" t="inlineStr">
+        <is>
+          <t>Cover Drive</t>
+        </is>
+      </c>
+      <c r="S241" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>Northern Cape Heat</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>Kimberley Oval</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>End 1</t>
+        </is>
+      </c>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>S Stolk</t>
+        </is>
+      </c>
+      <c r="J242" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K242" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="L242" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M242" t="inlineStr">
+        <is>
+          <t>Outside Leg</t>
+        </is>
+      </c>
+      <c r="N242" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="O242" t="n">
+        <v>0</v>
+      </c>
+      <c r="P242" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="R242" t="inlineStr">
+        <is>
+          <t>Front Foot Defense</t>
+        </is>
+      </c>
+      <c r="S242" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>Northern Cape Heat</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>Kimberley Oval</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>End 1</t>
+        </is>
+      </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>S Stolk</t>
+        </is>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K243" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="L243" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M243" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="N243" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="O243" t="n">
+        <v>5</v>
+      </c>
+      <c r="P243" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="Q243" t="inlineStr">
+        <is>
+          <t>Cover</t>
+        </is>
+      </c>
+      <c r="R243" t="inlineStr">
+        <is>
+          <t>Front Foot Defense</t>
+        </is>
+      </c>
+      <c r="S243" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>Northern Cape Heat</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>Kimberley Oval</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>End 1</t>
+        </is>
+      </c>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>L Doherty</t>
+        </is>
+      </c>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K244" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="L244" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M244" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="N244" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="O244" t="n">
+        <v>0</v>
+      </c>
+      <c r="P244" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="R244" t="inlineStr">
+        <is>
+          <t>Cover Drive</t>
+        </is>
+      </c>
+      <c r="S244" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>Northern Cape Heat</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>Kimberley Oval</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>End 1</t>
+        </is>
+      </c>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>L Doherty</t>
+        </is>
+      </c>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K245" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="L245" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M245" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="N245" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="O245" t="n">
+        <v>0</v>
+      </c>
+      <c r="P245" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="R245" t="inlineStr">
+        <is>
+          <t>Cover Drive</t>
+        </is>
+      </c>
+      <c r="S245" t="inlineStr">
+        <is>
+          <t>Miss</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>Northern Cape Heat</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>Kimberley Oval</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>End 1</t>
+        </is>
+      </c>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>L Doherty</t>
+        </is>
+      </c>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K246" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="L246" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M246" t="inlineStr">
+        <is>
+          <t>Outside Leg</t>
+        </is>
+      </c>
+      <c r="N246" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="O246" t="n">
+        <v>1</v>
+      </c>
+      <c r="P246" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="Q246" t="inlineStr">
+        <is>
+          <t>Fine Leg</t>
+        </is>
+      </c>
+      <c r="R246" t="inlineStr">
+        <is>
+          <t>Back Foot Flick</t>
+        </is>
+      </c>
+      <c r="S246" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>Northern Cape Heat</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>Kimberley Oval</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>End 1</t>
+        </is>
+      </c>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>S Stolk</t>
+        </is>
+      </c>
+      <c r="J247" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K247" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="L247" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M247" t="inlineStr">
+        <is>
+          <t>Off Stump</t>
+        </is>
+      </c>
+      <c r="N247" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="O247" t="n">
+        <v>2</v>
+      </c>
+      <c r="P247" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="Q247" t="inlineStr">
+        <is>
+          <t>Cow Corner</t>
+        </is>
+      </c>
+      <c r="R247" t="inlineStr">
+        <is>
+          <t>Back Foot Flick</t>
+        </is>
+      </c>
+      <c r="S247" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>Northern Cape Heat</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>Kimberley Oval</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>End 1</t>
+        </is>
+      </c>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>S Stolk</t>
+        </is>
+      </c>
+      <c r="J248" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K248" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="L248" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M248" t="inlineStr">
+        <is>
+          <t>Leg Stump</t>
+        </is>
+      </c>
+      <c r="N248" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="O248" t="n">
+        <v>1</v>
+      </c>
+      <c r="P248" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="Q248" t="inlineStr">
+        <is>
+          <t>Square Leg</t>
+        </is>
+      </c>
+      <c r="R248" t="inlineStr">
+        <is>
+          <t>Pull</t>
+        </is>
+      </c>
+      <c r="S248" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>Northern Cape Heat</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>Kimberley Oval</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>End 1</t>
+        </is>
+      </c>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>N Yikha</t>
+        </is>
+      </c>
+      <c r="J249" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K249" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="L249" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M249" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="N249" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="O249" t="n">
+        <v>0</v>
+      </c>
+      <c r="P249" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="R249" t="inlineStr">
+        <is>
+          <t>Cut</t>
+        </is>
+      </c>
+      <c r="S249" t="inlineStr">
+        <is>
+          <t>Miss</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>Northern Cape Heat</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>Kimberley Oval</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>End 1</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>N Yikha</t>
+        </is>
+      </c>
+      <c r="J250" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K250" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="L250" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M250" t="inlineStr">
+        <is>
+          <t>Middle Stump</t>
+        </is>
+      </c>
+      <c r="N250" t="inlineStr">
+        <is>
+          <t>Yorker</t>
+        </is>
+      </c>
+      <c r="O250" t="n">
+        <v>1</v>
+      </c>
+      <c r="P250" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="Q250" t="inlineStr">
+        <is>
+          <t>Cover</t>
+        </is>
+      </c>
+      <c r="R250" t="inlineStr">
+        <is>
+          <t>Dig Out</t>
+        </is>
+      </c>
+      <c r="S250" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>Northern Cape Heat</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>Kimberley Oval</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>End 1</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>S Stolk</t>
+        </is>
+      </c>
+      <c r="J251" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K251" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="L251" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M251" t="inlineStr">
+        <is>
+          <t>Middle Stump</t>
+        </is>
+      </c>
+      <c r="N251" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="O251" t="n">
+        <v>6</v>
+      </c>
+      <c r="P251" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="Q251" t="inlineStr">
+        <is>
+          <t>Mid Wicket</t>
+        </is>
+      </c>
+      <c r="R251" t="inlineStr">
+        <is>
+          <t>Pull</t>
+        </is>
+      </c>
+      <c r="S251" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>Northern Cape Heat</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>Kimberley Oval</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>End 1</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>S Stolk</t>
+        </is>
+      </c>
+      <c r="J252" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K252" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="L252" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M252" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="N252" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="O252" t="n">
+        <v>6</v>
+      </c>
+      <c r="P252" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="Q252" t="inlineStr">
+        <is>
+          <t>Extra Cover</t>
+        </is>
+      </c>
+      <c r="R252" t="inlineStr">
+        <is>
+          <t>Lofted Cover Drive</t>
+        </is>
+      </c>
+      <c r="S252" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>Northern Cape Heat</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>Kimberley Oval</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>End 2</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>K Jacobs</t>
+        </is>
+      </c>
+      <c r="J253" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K253" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="L253" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M253" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="N253" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="O253" t="n">
+        <v>1</v>
+      </c>
+      <c r="P253" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="Q253" t="inlineStr">
+        <is>
+          <t>Cow Corner</t>
+        </is>
+      </c>
+      <c r="R253" t="inlineStr">
+        <is>
+          <t>Pull</t>
+        </is>
+      </c>
+      <c r="S253" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>Northern Cape Heat</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>Kimberley Oval</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>End 2</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>T Isaac</t>
+        </is>
+      </c>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>Left</t>
+        </is>
+      </c>
+      <c r="K254" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="L254" t="inlineStr">
+        <is>
+          <t>Around</t>
+        </is>
+      </c>
+      <c r="M254" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="N254" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="O254" t="n">
+        <v>1</v>
+      </c>
+      <c r="P254" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="Q254" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="R254" t="inlineStr">
+        <is>
+          <t>Pull</t>
+        </is>
+      </c>
+      <c r="S254" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>Northern Cape Heat</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>Kimberley Oval</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>End 2</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>K Jacobs</t>
+        </is>
+      </c>
+      <c r="J255" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K255" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="L255" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M255" t="inlineStr">
+        <is>
+          <t>Off Stump</t>
+        </is>
+      </c>
+      <c r="N255" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="O255" t="inlineStr">
+        <is>
+          <t>Wicket</t>
+        </is>
+      </c>
+      <c r="P255" t="inlineStr">
+        <is>
+          <t>Caught</t>
+        </is>
+      </c>
+      <c r="Q255" t="inlineStr">
+        <is>
+          <t>Keeper</t>
+        </is>
+      </c>
+      <c r="R255" t="inlineStr">
+        <is>
+          <t>Reverse Scoop</t>
+        </is>
+      </c>
+      <c r="S255" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>Northern Cape Heat</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>Kimberley Oval</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>End 2</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>T Ntuli</t>
+        </is>
+      </c>
+      <c r="J256" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K256" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="L256" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M256" t="inlineStr">
+        <is>
+          <t>Outside Leg</t>
+        </is>
+      </c>
+      <c r="N256" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="O256" t="n">
+        <v>1</v>
+      </c>
+      <c r="P256" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="Q256" t="inlineStr">
+        <is>
+          <t>Square Leg</t>
+        </is>
+      </c>
+      <c r="R256" t="inlineStr">
+        <is>
+          <t>Pull</t>
+        </is>
+      </c>
+      <c r="S256" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>Northern Cape Heat</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>Kimberley Oval</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>End 2</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>T Isaac</t>
+        </is>
+      </c>
+      <c r="J257" t="inlineStr">
+        <is>
+          <t>Left</t>
+        </is>
+      </c>
+      <c r="K257" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="L257" t="inlineStr">
+        <is>
+          <t>Around</t>
+        </is>
+      </c>
+      <c r="M257" t="inlineStr">
+        <is>
+          <t>Outside Leg</t>
+        </is>
+      </c>
+      <c r="N257" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="O257" t="n">
+        <v>1</v>
+      </c>
+      <c r="P257" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="Q257" t="inlineStr">
+        <is>
+          <t>Fine Leg</t>
+        </is>
+      </c>
+      <c r="R257" t="inlineStr">
+        <is>
+          <t>Pull</t>
+        </is>
+      </c>
+      <c r="S257" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>YesPlay Pro20 Cup</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>Limpopo Impalas</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>Northern Cape Heat</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>Kimberley Oval</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>End 2</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>T Ntuli</t>
+        </is>
+      </c>
+      <c r="J258" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="K258" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="L258" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="M258" t="inlineStr">
+        <is>
+          <t>Middle Stump</t>
+        </is>
+      </c>
+      <c r="N258" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="O258" t="n">
+        <v>2</v>
+      </c>
+      <c r="P258" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="Q258" t="inlineStr">
+        <is>
+          <t>Mid Wicket</t>
+        </is>
+      </c>
+      <c r="R258" t="inlineStr">
+        <is>
+          <t>Hack</t>
+        </is>
+      </c>
+      <c r="S258" t="inlineStr">
         <is>
           <t>Contact</t>
         </is>

</xml_diff>

<commit_message>
Classify all 13 opposition bowlers' types
Via the Assign Bowler Types tool - every bowler Thomas has faced so
far now has a type recorded.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/raw/Mayes_Bowling_Batting.xlsx
+++ b/backend/data/raw/Mayes_Bowling_Batting.xlsx
@@ -27305,6 +27305,11 @@
           <t>H Coetzer</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Right Arm Medium</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr">
         <is>
           <t>Off Stump</t>
@@ -27384,6 +27389,11 @@
           <t>A Mhletywa</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>Outside Leg</t>
@@ -27463,6 +27473,11 @@
           <t>A Mhletywa</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L4" t="inlineStr">
         <is>
           <t>Outside Leg</t>
@@ -27542,6 +27557,11 @@
           <t>H Coetzer</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Right Arm Medium</t>
+        </is>
+      </c>
       <c r="L5" t="inlineStr">
         <is>
           <t>Off Stump</t>
@@ -27621,6 +27641,11 @@
           <t>A Mhletywa</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>Leg Stump</t>
@@ -27700,6 +27725,11 @@
           <t>A Mhletywa</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L7" t="inlineStr">
         <is>
           <t>Middle Stump</t>
@@ -27779,6 +27809,11 @@
           <t>A Mhletywa</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L8" t="inlineStr">
         <is>
           <t>Leg Stump</t>
@@ -27858,6 +27893,11 @@
           <t>A Mhletywa</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>Middle Stump</t>
@@ -27937,6 +27977,11 @@
           <t>S Langa</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Right Arm Medium</t>
+        </is>
+      </c>
       <c r="L10" t="inlineStr">
         <is>
           <t>Leg Stump</t>
@@ -28016,6 +28061,11 @@
           <t>S Langa</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Right Arm Medium</t>
+        </is>
+      </c>
       <c r="L11" t="inlineStr">
         <is>
           <t>Leg Stump</t>
@@ -28095,6 +28145,11 @@
           <t>S Langa</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Right Arm Medium</t>
+        </is>
+      </c>
       <c r="L12" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -28174,6 +28229,11 @@
           <t>S Langa</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Right Arm Medium</t>
+        </is>
+      </c>
       <c r="L13" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -28253,6 +28313,11 @@
           <t>A Mhletywa</t>
         </is>
       </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L14" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -28332,6 +28397,11 @@
           <t>A Mhletywa</t>
         </is>
       </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L15" t="inlineStr">
         <is>
           <t>Leg Stump</t>
@@ -28411,6 +28481,11 @@
           <t>A Mhletywa</t>
         </is>
       </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L16" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -28490,6 +28565,11 @@
           <t>S Langa</t>
         </is>
       </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Right Arm Medium</t>
+        </is>
+      </c>
       <c r="L17" t="inlineStr">
         <is>
           <t>Leg Stump</t>
@@ -28569,6 +28649,11 @@
           <t>S Langa</t>
         </is>
       </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Right Arm Medium</t>
+        </is>
+      </c>
       <c r="L18" t="inlineStr">
         <is>
           <t>Off Stump</t>
@@ -28648,6 +28733,11 @@
           <t>S Langa</t>
         </is>
       </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Right Arm Medium</t>
+        </is>
+      </c>
       <c r="L19" t="inlineStr">
         <is>
           <t>Outside Leg</t>
@@ -28727,6 +28817,11 @@
           <t>S Langa</t>
         </is>
       </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Right Arm Medium</t>
+        </is>
+      </c>
       <c r="L20" t="inlineStr">
         <is>
           <t>Wide</t>
@@ -28806,6 +28901,11 @@
           <t>T Ntini</t>
         </is>
       </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L21" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -28885,6 +28985,11 @@
           <t>T Ntini</t>
         </is>
       </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L22" t="inlineStr">
         <is>
           <t>Middle Stump</t>
@@ -28964,6 +29069,11 @@
           <t>S Langa</t>
         </is>
       </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Right Arm Medium</t>
+        </is>
+      </c>
       <c r="L23" t="inlineStr">
         <is>
           <t>Outside Leg</t>
@@ -29043,6 +29153,11 @@
           <t>S Langa</t>
         </is>
       </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Right Arm Medium</t>
+        </is>
+      </c>
       <c r="L24" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -29122,6 +29237,11 @@
           <t>S Langa</t>
         </is>
       </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Right Arm Medium</t>
+        </is>
+      </c>
       <c r="L25" t="inlineStr">
         <is>
           <t>Middle Stump</t>
@@ -29201,6 +29321,11 @@
           <t>T Ntini</t>
         </is>
       </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L26" t="inlineStr">
         <is>
           <t>Middle Stump</t>
@@ -29280,6 +29405,11 @@
           <t>T Ntini</t>
         </is>
       </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L27" t="inlineStr">
         <is>
           <t>Middle Stump</t>
@@ -29359,6 +29489,11 @@
           <t>T Ntini</t>
         </is>
       </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L28" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -29438,6 +29573,11 @@
           <t>T Ntini</t>
         </is>
       </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L29" t="inlineStr">
         <is>
           <t>Wide</t>
@@ -29517,6 +29657,11 @@
           <t>S Langa</t>
         </is>
       </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Right Arm Medium</t>
+        </is>
+      </c>
       <c r="L30" t="inlineStr">
         <is>
           <t>Outside Leg</t>
@@ -29596,6 +29741,11 @@
           <t>S Langa</t>
         </is>
       </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Right Arm Medium</t>
+        </is>
+      </c>
       <c r="L31" t="inlineStr">
         <is>
           <t>Leg Stump</t>
@@ -29675,6 +29825,11 @@
           <t>T Ntini</t>
         </is>
       </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L32" t="inlineStr">
         <is>
           <t>Wide</t>
@@ -29754,6 +29909,11 @@
           <t>T Ntini</t>
         </is>
       </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L33" t="inlineStr">
         <is>
           <t>Leg Stump</t>
@@ -29833,6 +29993,11 @@
           <t>T Ntini</t>
         </is>
       </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L34" t="inlineStr">
         <is>
           <t>Wide</t>
@@ -29912,6 +30077,11 @@
           <t>N Smith</t>
         </is>
       </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L35" t="inlineStr">
         <is>
           <t>Leg Stump</t>
@@ -29991,6 +30161,11 @@
           <t>Z Foulkes</t>
         </is>
       </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L36" t="inlineStr">
         <is>
           <t>Leg Stump</t>
@@ -30070,6 +30245,11 @@
           <t>Z Foulkes</t>
         </is>
       </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L37" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -30149,6 +30329,11 @@
           <t>Z Foulkes</t>
         </is>
       </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L38" t="inlineStr">
         <is>
           <t>Middle Stump</t>
@@ -30228,6 +30413,11 @@
           <t>Z Foulkes</t>
         </is>
       </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L39" t="inlineStr">
         <is>
           <t>Middle Stump</t>
@@ -30307,6 +30497,11 @@
           <t>N Smith</t>
         </is>
       </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L40" t="inlineStr">
         <is>
           <t>Off Stump</t>
@@ -30386,6 +30581,11 @@
           <t>N Smith</t>
         </is>
       </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L41" t="inlineStr">
         <is>
           <t>Leg Stump</t>
@@ -30465,6 +30665,11 @@
           <t>B Tickner</t>
         </is>
       </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L42" t="inlineStr">
         <is>
           <t>Middle Stump</t>
@@ -30546,6 +30751,11 @@
           <t>B Tickner</t>
         </is>
       </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L43" t="inlineStr">
         <is>
           <t>Off Stump</t>
@@ -30625,6 +30835,11 @@
           <t>B Tickner</t>
         </is>
       </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L44" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -30704,6 +30919,11 @@
           <t>B Tickner</t>
         </is>
       </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L45" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -30783,6 +31003,11 @@
           <t>B Tickner</t>
         </is>
       </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L46" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -30862,6 +31087,11 @@
           <t>N Smith</t>
         </is>
       </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L47" t="inlineStr">
         <is>
           <t>Middle Stump</t>
@@ -30941,6 +31171,11 @@
           <t>N Smith</t>
         </is>
       </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L48" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -31020,6 +31255,11 @@
           <t>N Smith</t>
         </is>
       </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L49" t="inlineStr">
         <is>
           <t>Middle Stump</t>
@@ -31099,6 +31339,11 @@
           <t>N Smith</t>
         </is>
       </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L50" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -31178,6 +31423,11 @@
           <t>N Smith</t>
         </is>
       </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L51" t="inlineStr">
         <is>
           <t>Leg Stump</t>
@@ -31257,6 +31507,11 @@
           <t>N Smith</t>
         </is>
       </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L52" t="inlineStr">
         <is>
           <t>Middle Stump</t>
@@ -31336,6 +31591,11 @@
           <t>B Tickner</t>
         </is>
       </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L53" t="inlineStr">
         <is>
           <t>Middle Stump</t>
@@ -31415,6 +31675,11 @@
           <t>N Smith</t>
         </is>
       </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L54" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -31494,6 +31759,11 @@
           <t>N Smith</t>
         </is>
       </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L55" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -31575,6 +31845,11 @@
           <t>H Coetzer</t>
         </is>
       </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Right Arm Medium</t>
+        </is>
+      </c>
       <c r="L56" t="inlineStr">
         <is>
           <t>Wide</t>
@@ -31654,6 +31929,11 @@
           <t>N Smith</t>
         </is>
       </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L57" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -31733,6 +32013,11 @@
           <t>B Tickner</t>
         </is>
       </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L58" t="inlineStr">
         <is>
           <t>Outside Leg</t>
@@ -31812,6 +32097,11 @@
           <t>B Tickner</t>
         </is>
       </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L59" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -31891,6 +32181,11 @@
           <t>B Tickner</t>
         </is>
       </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L60" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -31970,6 +32265,11 @@
           <t>B Tickner</t>
         </is>
       </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L61" t="inlineStr">
         <is>
           <t>Leg Stump</t>
@@ -32049,6 +32349,11 @@
           <t>B Tickner</t>
         </is>
       </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L62" t="inlineStr">
         <is>
           <t>Leg Stump</t>
@@ -32128,6 +32433,11 @@
           <t>B Tickner</t>
         </is>
       </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L63" t="inlineStr">
         <is>
           <t>Leg Stump</t>
@@ -32207,6 +32517,11 @@
           <t>B Tickner</t>
         </is>
       </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L64" t="inlineStr">
         <is>
           <t>Leg Stump</t>
@@ -32286,6 +32601,11 @@
           <t>B Tickner</t>
         </is>
       </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L65" t="inlineStr">
         <is>
           <t>Leg Stump</t>
@@ -32365,6 +32685,11 @@
           <t>B Tickner</t>
         </is>
       </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L66" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -32444,6 +32769,11 @@
           <t>N Smith</t>
         </is>
       </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L67" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -32523,6 +32853,11 @@
           <t>N Smith</t>
         </is>
       </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L68" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -32602,6 +32937,11 @@
           <t>N Smith</t>
         </is>
       </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L69" t="inlineStr">
         <is>
           <t>Outside Leg</t>
@@ -32681,6 +33021,11 @@
           <t>N Smith</t>
         </is>
       </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L70" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -32760,6 +33105,11 @@
           <t>H Coetzer</t>
         </is>
       </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>Right Arm Medium</t>
+        </is>
+      </c>
       <c r="L71" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -32839,6 +33189,11 @@
           <t>S Langa</t>
         </is>
       </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>Right Arm Medium</t>
+        </is>
+      </c>
       <c r="L72" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -32918,6 +33273,11 @@
           <t>N Smith</t>
         </is>
       </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L73" t="inlineStr">
         <is>
           <t>Outside Leg</t>
@@ -32997,6 +33357,11 @@
           <t>N Smith</t>
         </is>
       </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L74" t="inlineStr">
         <is>
           <t>Outside Leg</t>
@@ -33076,6 +33441,11 @@
           <t>S Kaber</t>
         </is>
       </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>Left Arm Wrist Spin</t>
+        </is>
+      </c>
       <c r="L75" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -33152,6 +33522,11 @@
           <t>T Luus</t>
         </is>
       </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L76" t="inlineStr">
         <is>
           <t>Wide</t>
@@ -33226,6 +33601,11 @@
           <t>T Luus</t>
         </is>
       </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L77" t="inlineStr">
         <is>
           <t>Leg Stump</t>
@@ -33302,6 +33682,11 @@
           <t>L Alder</t>
         </is>
       </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>Left Arm Finger Spin</t>
+        </is>
+      </c>
       <c r="L78" t="inlineStr">
         <is>
           <t>Middle Stump</t>
@@ -33381,6 +33766,11 @@
           <t>L Alder</t>
         </is>
       </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>Left Arm Finger Spin</t>
+        </is>
+      </c>
       <c r="L79" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -33455,6 +33845,11 @@
           <t>L Alder</t>
         </is>
       </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>Left Arm Finger Spin</t>
+        </is>
+      </c>
       <c r="L80" t="inlineStr">
         <is>
           <t>Middle Stump</t>
@@ -33529,6 +33924,11 @@
           <t>E Kitshini</t>
         </is>
       </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>Left Arm Finger Spin</t>
+        </is>
+      </c>
       <c r="L81" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -33603,6 +34003,11 @@
           <t>E Kitshini</t>
         </is>
       </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>Left Arm Finger Spin</t>
+        </is>
+      </c>
       <c r="L82" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -33677,6 +34082,11 @@
           <t>E Kitshini</t>
         </is>
       </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>Left Arm Finger Spin</t>
+        </is>
+      </c>
       <c r="L83" t="inlineStr">
         <is>
           <t>Middle Stump</t>
@@ -33751,6 +34161,11 @@
           <t>E Kitshini</t>
         </is>
       </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>Left Arm Finger Spin</t>
+        </is>
+      </c>
       <c r="L84" t="inlineStr">
         <is>
           <t>Off Stump</t>
@@ -33825,6 +34240,11 @@
           <t>E Kitshini</t>
         </is>
       </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>Left Arm Finger Spin</t>
+        </is>
+      </c>
       <c r="L85" t="inlineStr">
         <is>
           <t>Leg Stump</t>
@@ -33899,6 +34319,11 @@
           <t>L Sadler</t>
         </is>
       </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L86" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -33978,6 +34403,11 @@
           <t>L Sadler</t>
         </is>
       </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L87" t="inlineStr">
         <is>
           <t>Off Stump</t>
@@ -34057,6 +34487,11 @@
           <t>L Sadler</t>
         </is>
       </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L88" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -34136,6 +34571,11 @@
           <t>B Cele</t>
         </is>
       </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>Right Arm Medium</t>
+        </is>
+      </c>
       <c r="L89" t="inlineStr">
         <is>
           <t>Off Stump</t>
@@ -34215,6 +34655,11 @@
           <t>B Cele</t>
         </is>
       </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>Right Arm Medium</t>
+        </is>
+      </c>
       <c r="L90" t="inlineStr">
         <is>
           <t>Wide</t>
@@ -34289,6 +34734,11 @@
           <t>L Sadler</t>
         </is>
       </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L91" t="inlineStr">
         <is>
           <t>Channel</t>
@@ -34368,6 +34818,11 @@
           <t>L Sadler</t>
         </is>
       </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L92" t="inlineStr">
         <is>
           <t>Wide</t>
@@ -34447,6 +34902,11 @@
           <t>L Sadler</t>
         </is>
       </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L93" t="inlineStr">
         <is>
           <t>Leg Stump</t>
@@ -34526,6 +34986,11 @@
           <t>L Sadler</t>
         </is>
       </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Right Arm Fast</t>
+        </is>
+      </c>
       <c r="L94" t="inlineStr">
         <is>
           <t>Wide</t>
@@ -34603,6 +35068,11 @@
       <c r="J95" t="inlineStr">
         <is>
           <t>B Cele</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>Right Arm Medium</t>
         </is>
       </c>
       <c r="L95" t="inlineStr">

</xml_diff>

<commit_message>
Add wicket explanation for the Northern Cape Heat match (19.3, K Jacobs)
Caught at Keeper - was blank.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/raw/Mayes_Bowling_Batting.xlsx
+++ b/backend/data/raw/Mayes_Bowling_Batting.xlsx
@@ -24545,6 +24545,11 @@
           <t>Edge</t>
         </is>
       </c>
+      <c r="T255" t="inlineStr">
+        <is>
+          <t>Caught at Keeper</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" s="2" t="n">

</xml_diff>